<commit_message>
feat(posy): implement fresh-chain simplified consensus
</commit_message>
<xml_diff>
--- a/launch/PoSy_Consensus_Parameter_Control_Workbook_v3_PROPOSAL.xlsx
+++ b/launch/PoSy_Consensus_Parameter_Control_Workbook_v3_PROPOSAL.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="1" r:id="Rf16951124e194511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validator Weights" sheetId="2" r:id="R866c9a9f5a1d4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter Register" sheetId="3" r:id="Ref043948b20c49e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activation Checklist" sheetId="4" r:id="Rc9e2f70caeb94a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="1" r:id="R69432832c8944fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validator Weights" sheetId="2" r:id="Rbcdfb76a721648ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter Register" sheetId="3" r:id="Rc71fb7aa8b604b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activation Checklist" sheetId="4" r:id="Raeec1174fb284224"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0.00%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -59,8 +59,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243B53"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +92,41 @@
         <x:fgColor rgb="FFFFF3CD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF102A43"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF102A43"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF102A43"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -94,7 +134,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -195,6 +235,53 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -438,7 +525,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>PROPOSAL ONLY — not governance-approved, not activated, and not launch-qualified. Existing finalized PoSy v2.2 bytes and root remain unchanged.</x:v>
+        <x:v>PROPOSAL ONLY — fresh block-zero Chain 1266 / Testnet-v3 PoSy source. Not governance-approved, release-authorized, activated, or launch-qualified.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -507,7 +594,7 @@
         <x:v>Parameter Register</x:v>
       </x:c>
       <x:c r="H5" s="14" t="str">
-        <x:v>No mixed v2.2/v3 objects</x:v>
+        <x:v>Retired-chain artifacts are rejected as P3 inputs</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60" hidden="0" customHeight="1">
@@ -524,7 +611,7 @@
         <x:v>PROPOSED</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
-        <x:v>Activation epoch</x:v>
+        <x:v>Fresh Genesis epoch 0 / height 1</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
         <x:v>Consensus Engineering</x:v>
@@ -776,25 +863,25 @@
         <x:v>ETDAG boundary</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Preserved</x:v>
+        <x:v>Governed and separated</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>BOC/reveal/protected execution remain separate</x:v>
+        <x:v>Parameter, fee, and membership-anchor commitments</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
-        <x:v>PRESERVED</x:v>
+        <x:v>PROPOSED</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>Existing activation gates</x:v>
+        <x:v>Verified V4 release approval</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
         <x:v>ETDAG Engineering</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>POSY-00D</x:v>
+        <x:v>ETDAG governance inputs</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>ETDAG never finalizes blocks</x:v>
+        <x:v>No ungoverned P3 fallback</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" hidden="0" customHeight="1">
@@ -805,7 +892,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:f>'Activation Checklist'!B22</x:f>
+        <x:f>'Activation Checklist'!B25</x:f>
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
@@ -861,7 +948,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>These five rows are initial-activation inputs only. Later epochs use a newly finalized frozen topology and dynamically derived quorum. Replace placeholders only with approved public records; never add private keys, credentials, or host secrets.</x:v>
+        <x:v>Initial epoch only: posy-validator-01..05 map to synergy-val2..6. Later epochs use a governed dynamic topology. Public identifiers and proposed weights only; never place keys, credentials, or host secrets here.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -893,7 +980,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="30" t="str">
-        <x:v>Validator Placeholder</x:v>
+        <x:v>Canonical Validator ID</x:v>
       </x:c>
       <x:c r="B5" s="30" t="str">
         <x:v>Active</x:v>
@@ -919,7 +1006,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="14" t="str">
-        <x:v>VALIDATOR-1-PUBLIC-ID-TBD</x:v>
+        <x:v>posy-validator-01</x:v>
       </x:c>
       <x:c r="B6" s="20" t="b">
         <x:v>1</x:v>
@@ -950,7 +1037,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
-        <x:v>VALIDATOR-2-PUBLIC-ID-TBD</x:v>
+        <x:v>posy-validator-02</x:v>
       </x:c>
       <x:c r="B7" s="20" t="b">
         <x:v>1</x:v>
@@ -981,7 +1068,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>VALIDATOR-3-PUBLIC-ID-TBD</x:v>
+        <x:v>posy-validator-03</x:v>
       </x:c>
       <x:c r="B8" s="20" t="b">
         <x:v>1</x:v>
@@ -1012,7 +1099,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>VALIDATOR-4-PUBLIC-ID-TBD</x:v>
+        <x:v>posy-validator-04</x:v>
       </x:c>
       <x:c r="B9" s="20" t="b">
         <x:v>1</x:v>
@@ -1043,7 +1130,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>VALIDATOR-5-PUBLIC-ID-TBD</x:v>
+        <x:v>posy-validator-05</x:v>
       </x:c>
       <x:c r="B10" s="20" t="b">
         <x:v>1</x:v>
@@ -1303,7 +1390,7 @@
         <x:v>proposal_parameter_root</x:v>
       </x:c>
       <x:c r="D8" s="15" t="str">
-        <x:v>2c8be6837fa49c160887cc1fcf2b741eadd72172bdeed27c9645c08ebe88be5fb562ca82e89af7cbe821157aba6d0e20a7727f0ff9e191a14dff5744fd4de101</x:v>
+        <x:v>91bbdd0101d5a6e9c6e72a5cc1160e85c074573f45b2a460d0b1487c9097b07504340768ff65365ccded5e5e96483ccb8cac00d025a457d8c1d4ee2fb547ba42</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
         <x:v>SHA3-512 of exact canonical manifest bytes</x:v>
@@ -1315,7 +1402,7 @@
         <x:v>PROPOSED</x:v>
       </x:c>
       <x:c r="H8" s="14" t="str">
-        <x:v>proposal verification record</x:v>
+        <x:v>TESTNET_V3_POSY_SIMPLIFIED_PARAMETER_PROPOSAL_VERIFICATION.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1862,7 +1949,7 @@
         <x:v>PROPOSED</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>five-process state-machine harness</x:v>
+        <x:v>five-node state-machine and production-driver harnesses</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -1928,10 +2015,10 @@
         <x:v>activation_epoch</x:v>
       </x:c>
       <x:c r="D32" s="15" t="str">
-        <x:v>TBD</x:v>
+        <x:v>null while proposed; 0 when FINALIZED</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>Finalized governance input</x:v>
+        <x:v>Fresh Genesis epoch is fixed and never migrated</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>Protocol</x:v>
@@ -1940,7 +2027,7 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>migration runbook</x:v>
+        <x:v>manifest schema / Genesis activation loader</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -1954,10 +2041,10 @@
         <x:v>activation_height</x:v>
       </x:c>
       <x:c r="D33" s="15" t="str">
-        <x:v>TBD</x:v>
+        <x:v>null while proposed; 1 when FINALIZED</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
-        <x:v>Exact epoch boundary</x:v>
+        <x:v>First consensus block follows block-zero Genesis</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
         <x:v>Protocol</x:v>
@@ -1966,7 +2053,241 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>migration runbook</x:v>
+        <x:v>manifest schema / Genesis activation loader</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="28" customHeight="1">
+      <x:c r="A34" s="33" t="str">
+        <x:v>ID-304</x:v>
+      </x:c>
+      <x:c r="B34" s="33" t="str">
+        <x:v>Identity</x:v>
+      </x:c>
+      <x:c r="C34" s="33" t="str">
+        <x:v>chain_id</x:v>
+      </x:c>
+      <x:c r="D34" s="44" t="n">
+        <x:v>1266</x:v>
+      </x:c>
+      <x:c r="E34" s="33" t="str">
+        <x:v>Exact integer</x:v>
+      </x:c>
+      <x:c r="F34" s="33" t="str">
+        <x:v>Protocol</x:v>
+      </x:c>
+      <x:c r="G34" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H34" s="33" t="str">
+        <x:v>parameter schema / genesis.rs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="28" customHeight="1">
+      <x:c r="A35" s="33" t="str">
+        <x:v>ID-305</x:v>
+      </x:c>
+      <x:c r="B35" s="33" t="str">
+        <x:v>Identity</x:v>
+      </x:c>
+      <x:c r="C35" s="33" t="str">
+        <x:v>network_id</x:v>
+      </x:c>
+      <x:c r="D35" s="44" t="str">
+        <x:v>testnet</x:v>
+      </x:c>
+      <x:c r="E35" s="33" t="str">
+        <x:v>Canonical technical environment ID</x:v>
+      </x:c>
+      <x:c r="F35" s="33" t="str">
+        <x:v>Protocol</x:v>
+      </x:c>
+      <x:c r="G35" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H35" s="33" t="str">
+        <x:v>parameter schema / genesis.rs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="28" customHeight="1">
+      <x:c r="A36" s="33" t="str">
+        <x:v>ID-306</x:v>
+      </x:c>
+      <x:c r="B36" s="33" t="str">
+        <x:v>Identity</x:v>
+      </x:c>
+      <x:c r="C36" s="33" t="str">
+        <x:v>release_id</x:v>
+      </x:c>
+      <x:c r="D36" s="44" t="str">
+        <x:v>testnet-v3</x:v>
+      </x:c>
+      <x:c r="E36" s="33" t="str">
+        <x:v>Human release identifier</x:v>
+      </x:c>
+      <x:c r="F36" s="33" t="str">
+        <x:v>Protocol</x:v>
+      </x:c>
+      <x:c r="G36" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H36" s="33" t="str">
+        <x:v>parameter schema / genesis.rs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="28" customHeight="1">
+      <x:c r="A37" s="33" t="str">
+        <x:v>GEN-301</x:v>
+      </x:c>
+      <x:c r="B37" s="33" t="str">
+        <x:v>Genesis</x:v>
+      </x:c>
+      <x:c r="C37" s="33" t="str">
+        <x:v>activation_boundary</x:v>
+      </x:c>
+      <x:c r="D37" s="44" t="str">
+        <x:v>fresh_genesis_block_zero</x:v>
+      </x:c>
+      <x:c r="E37" s="33" t="str">
+        <x:v>No transition, replay, or retired state input</x:v>
+      </x:c>
+      <x:c r="F37" s="33" t="str">
+        <x:v>Security-sensitive</x:v>
+      </x:c>
+      <x:c r="G37" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H37" s="33" t="str">
+        <x:v>genesis.rs / prepare-fresh-posy-v3-genesis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="28" customHeight="1">
+      <x:c r="A38" s="33" t="str">
+        <x:v>GEN-302</x:v>
+      </x:c>
+      <x:c r="B38" s="33" t="str">
+        <x:v>Finality</x:v>
+      </x:c>
+      <x:c r="C38" s="33" t="str">
+        <x:v>genesis_finality_parent</x:v>
+      </x:c>
+      <x:c r="D38" s="44" t="str">
+        <x:v>typed non-QC parent</x:v>
+      </x:c>
+      <x:c r="E38" s="33" t="str">
+        <x:v>Block 1 names Genesis; block 2+ require QC parents</x:v>
+      </x:c>
+      <x:c r="F38" s="33" t="str">
+        <x:v>Security-sensitive</x:v>
+      </x:c>
+      <x:c r="G38" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H38" s="33" t="str">
+        <x:v>SimplifiedFinalityParent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="33" t="str">
+        <x:v>ETDAG-303</x:v>
+      </x:c>
+      <x:c r="B39" s="33" t="str">
+        <x:v>ETDAG</x:v>
+      </x:c>
+      <x:c r="C39" s="33" t="str">
+        <x:v>initial_etdag_activation</x:v>
+      </x:c>
+      <x:c r="D39" s="44" t="str">
+        <x:v>governed_genesis_binding_required</x:v>
+      </x:c>
+      <x:c r="E39" s="33" t="str">
+        <x:v>Fail closed without governed parameter and fee artifacts</x:v>
+      </x:c>
+      <x:c r="F39" s="33" t="str">
+        <x:v>Security-sensitive</x:v>
+      </x:c>
+      <x:c r="G39" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H39" s="33" t="str">
+        <x:v>etdag_governance.rs / role_runtime.rs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="33" t="str">
+        <x:v>ETDAG-304</x:v>
+      </x:c>
+      <x:c r="B40" s="33" t="str">
+        <x:v>ETDAG</x:v>
+      </x:c>
+      <x:c r="C40" s="33" t="str">
+        <x:v>release_commitments</x:v>
+      </x:c>
+      <x:c r="D40" s="44" t="str">
+        <x:v>parameter root + fee root + membership anchor</x:v>
+      </x:c>
+      <x:c r="E40" s="33" t="str">
+        <x:v>All three nonzero SHA3-512 commitments bound by V4 approval</x:v>
+      </x:c>
+      <x:c r="F40" s="33" t="str">
+        <x:v>Security-sensitive</x:v>
+      </x:c>
+      <x:c r="G40" s="33" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="H40" s="33" t="str">
+        <x:v>testnet_v3_release_approval.rs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="33" t="str">
+        <x:v>GOV-301</x:v>
+      </x:c>
+      <x:c r="B41" s="33" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="C41" s="33" t="str">
+        <x:v>release_approval_schema</x:v>
+      </x:c>
+      <x:c r="D41" s="44" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E41" s="33" t="str">
+        <x:v>V4 is the approval schema, not a chain version</x:v>
+      </x:c>
+      <x:c r="F41" s="33" t="str">
+        <x:v>Security-sensitive</x:v>
+      </x:c>
+      <x:c r="G41" s="33" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="H41" s="33" t="str">
+        <x:v>Core verifier / Address Engine signer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="33" t="str">
+        <x:v>ONB-301</x:v>
+      </x:c>
+      <x:c r="B42" s="33" t="str">
+        <x:v>Membership</x:v>
+      </x:c>
+      <x:c r="C42" s="33" t="str">
+        <x:v>validator_set_growth</x:v>
+      </x:c>
+      <x:c r="D42" s="44" t="str">
+        <x:v>dynamic finalized epoch transitions</x:v>
+      </x:c>
+      <x:c r="E42" s="33" t="str">
+        <x:v>Initial five is not a membership ceiling</x:v>
+      </x:c>
+      <x:c r="F42" s="33" t="str">
+        <x:v>Protocol</x:v>
+      </x:c>
+      <x:c r="G42" s="33" t="str">
+        <x:v>PROPOSED</x:v>
+      </x:c>
+      <x:c r="H42" s="33" t="str">
+        <x:v>transition.rs / activation.rs</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2088,22 +2409,22 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>Activation epoch/height declared</x:v>
+        <x:v>Fresh Genesis epoch/height fixed</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>SOURCE PASS</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>Finalized transition record</x:v>
+        <x:v>Schema requires epoch 0 and first consensus height 1 when finalized</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>migration package</x:v>
+        <x:v>parameter proposal/schema</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
         <x:v>Protocol Governance</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
-        <x:v>Remain posy/2.2</x:v>
+        <x:v>Refuse chain start</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -2249,22 +2570,22 @@
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>Five-process state-machine harness</x:v>
+        <x:v>Five-node state-machine and production-driver harnesses</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Five processes using production state/signing APIs; full node/P2P/ETDAG remains open</x:v>
+        <x:v>Both distinct harnesses pass with production state/signing APIs</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>runtime harness</x:v>
+        <x:v>runtime harness evidence</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
         <x:v>QA</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
-        <x:v>Do not claim node integration</x:v>
+        <x:v>Do not claim integration completion</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -2309,22 +2630,22 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Activation and onboarding transition rehearsal</x:v>
+        <x:v>Fresh Genesis and dynamic-onboarding rehearsal</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>Initial five share one boundary; later validators enter only through a finalized epoch transition</x:v>
+        <x:v>Initial five start from block zero; later validators join only through finalized epoch transitions</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>migration runbook</x:v>
+        <x:v>fresh-chain launch runbook</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
         <x:v>Validator Operations</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Abort before boundary</x:v>
+        <x:v>Abort before chain start</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -2367,18 +2688,78 @@
         <x:v>Launch remains blocked</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="26" t="str">
+    <x:row r="22" ht="32" hidden="0" customHeight="1">
+      <x:c r="A22" s="45" t="str">
+        <x:v>Governed ETDAG roots and membership anchor</x:v>
+      </x:c>
+      <x:c r="B22" s="48" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="C22" s="46" t="str">
+        <x:v>Nonzero canonical parameter root, fee root, and Genesis-bound anchor</x:v>
+      </x:c>
+      <x:c r="D22" s="46" t="str">
+        <x:v>ETDAG governance inputs / final candidate</x:v>
+      </x:c>
+      <x:c r="E22" s="46" t="str">
+        <x:v>ETDAG Engineering</x:v>
+      </x:c>
+      <x:c r="F22" s="46" t="str">
+        <x:v>Refuse release approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="32" customHeight="1">
+      <x:c r="A23" s="47" t="str">
+        <x:v>Frozen-governance V4 release approval</x:v>
+      </x:c>
+      <x:c r="B23" s="44" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="str">
+        <x:v>Verified ML-DSA-87 signature over the exact final candidate and all governed roots</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="str">
+        <x:v>signed release approval</x:v>
+      </x:c>
+      <x:c r="E23" s="47" t="str">
+        <x:v>Release Authority</x:v>
+      </x:c>
+      <x:c r="F23" s="47" t="str">
+        <x:v>Do not activate or publish Wallet trust</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="32" customHeight="1">
+      <x:c r="A24" s="47" t="str">
+        <x:v>Wallet public trust derivation</x:v>
+      </x:c>
+      <x:c r="B24" s="44" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>Registry values derived from the verified release and Wallet gate passes</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="str">
+        <x:v>Wallet release evidence</x:v>
+      </x:c>
+      <x:c r="E24" s="47" t="str">
+        <x:v>Wallet Release</x:v>
+      </x:c>
+      <x:c r="F24" s="47" t="str">
+        <x:v>Do not package or publish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="49" t="str">
         <x:v>Overall Activation Status</x:v>
       </x:c>
-      <x:c r="B22" s="26" t="str">
-        <x:f>IF(COUNTIF(B6:B21,"PASS")=ROWS(B6:B21),"PASS","BLOCKED")</x:f>
+      <x:c r="B25" s="49" t="str">
+        <x:f>IF(COUNTIF(B6:B24,"*PASS")=ROWS(B6:B24),"PASS","BLOCKED")</x:f>
         <x:v>BLOCKED</x:v>
       </x:c>
-      <x:c r="C22" s="14"/>
-      <x:c r="D22" s="14"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="14"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat(testnet-v3): complete PoSy release-readiness boundary
</commit_message>
<xml_diff>
--- a/launch/PoSy_Consensus_Parameter_Control_Workbook_v3_PROPOSAL.xlsx
+++ b/launch/PoSy_Consensus_Parameter_Control_Workbook_v3_PROPOSAL.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="1" r:id="R69432832c8944fa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validator Weights" sheetId="2" r:id="Rbcdfb76a721648ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter Register" sheetId="3" r:id="Rc71fb7aa8b604b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activation Checklist" sheetId="4" r:id="Raeec1174fb284224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="1" r:id="Rb89f6ccded4c4273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validator Weights" sheetId="2" r:id="R6d114ceca4074d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter Register" sheetId="3" r:id="Rbc68c1418c2b40c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activation Checklist" sheetId="4" r:id="R3911a65dda37457d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -948,7 +948,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>Initial epoch only: posy-validator-01..05 map to synergy-val2..6. Later epochs use a governed dynamic topology. Public identifiers and proposed weights only; never place keys, credentials, or host secrets here.</x:v>
+        <x:v>Initial epoch only: validator-02..validator-06 map to synergy-val2..synergy-val6. Later epochs use a governed dynamic topology. Public identifiers and proposed weights only; never place keys, credentials, or host secrets here.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -1006,7 +1006,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="14" t="str">
-        <x:v>posy-validator-01</x:v>
+        <x:v>validator-02</x:v>
       </x:c>
       <x:c r="B6" s="20" t="b">
         <x:v>1</x:v>
@@ -1037,7 +1037,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
-        <x:v>posy-validator-02</x:v>
+        <x:v>validator-03</x:v>
       </x:c>
       <x:c r="B7" s="20" t="b">
         <x:v>1</x:v>
@@ -1068,7 +1068,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>posy-validator-03</x:v>
+        <x:v>validator-04</x:v>
       </x:c>
       <x:c r="B8" s="20" t="b">
         <x:v>1</x:v>
@@ -1099,7 +1099,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>posy-validator-04</x:v>
+        <x:v>validator-05</x:v>
       </x:c>
       <x:c r="B9" s="20" t="b">
         <x:v>1</x:v>
@@ -1130,7 +1130,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>posy-validator-05</x:v>
+        <x:v>validator-06</x:v>
       </x:c>
       <x:c r="B10" s="20" t="b">
         <x:v>1</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
-        <x:v>Ratified POSY-00E and updated coordinated set</x:v>
+        <x:v>Ratified POSY-00E and updated simplified PoSy set</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
         <x:v>docs/posy-v3</x:v>

</xml_diff>